<commit_message>
Update with FTNIR results
</commit_message>
<xml_diff>
--- a/output/best_p_lipid_models.xlsx
+++ b/output/best_p_lipid_models.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean.rohan\Work\afsc\fatmeter\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C7614B-7DF5-4142-9198-25539D106311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E4836C-796F-4733-AC36-D55090AF8419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32865" yWindow="3675" windowWidth="21600" windowHeight="11295" xr2:uid="{0233C46D-F3A1-4536-8D9F-A4B59563ECFB}"/>
+    <workbookView xWindow="33315" yWindow="3300" windowWidth="21600" windowHeight="11295" xr2:uid="{0233C46D-F3A1-4536-8D9F-A4B59563ECFB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="16">
   <si>
     <t>common_name</t>
   </si>
@@ -80,16 +80,10 @@
     <t>liver_12</t>
   </si>
   <si>
-    <t>liver_6</t>
-  </si>
-  <si>
-    <t>liver_9</t>
-  </si>
-  <si>
-    <t>liver_17</t>
-  </si>
-  <si>
     <t>liver_18</t>
+  </si>
+  <si>
+    <t>liver_16</t>
   </si>
 </sst>
 </file>
@@ -492,7 +486,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -520,7 +514,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -548,7 +542,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -576,7 +570,7 @@
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>

</xml_diff>